<commit_message>
fix: preserve XTB operation and comment boundaries
</commit_message>
<xml_diff>
--- a/tests/Fixtures/Xtb/synthetic-xtb-statement.xlsx
+++ b/tests/Fixtures/Xtb/synthetic-xtb-statement.xlsx
@@ -85,7 +85,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>Stock purchase</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -119,7 +119,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>Stock sale</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">

</xml_diff>